<commit_message>
new script, new plots
</commit_message>
<xml_diff>
--- a/Python/Determinants_and_Elasticity_of_Czech_Export/Data/df.xlsx
+++ b/Python/Determinants_and_Elasticity_of_Czech_Export/Data/df.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petrchaloupek/00 Soubory pro R/MacroeconomicModeling/R/Diplomka/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petrchaloupek/00 Soubory pro R/MacroeconomicModeling/Python/Determinants_and_Elasticity_of_Czech_Export/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C0F7F2-67BD-5844-BB0A-58DE085B3495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92752E7D-459D-B34A-A82D-1EDCC768A6AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17160" xr2:uid="{9E3E9A4F-CC29-154C-B8BB-E88AAB0D6DA7}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17160" activeTab="2" xr2:uid="{9E3E9A4F-CC29-154C-B8BB-E88AAB0D6DA7}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="19">
   <si>
     <t>Date</t>
   </si>
@@ -94,7 +94,7 @@
     <t>ULC</t>
   </si>
   <si>
-    <t>log</t>
+    <t>y</t>
   </si>
 </sst>
 </file>
@@ -12259,294 +12259,294 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>List2!$C$2:$C$96</c:f>
+              <c:f>List2!$G$2:$G$96</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="95"/>
                 <c:pt idx="0">
-                  <c:v>5.4239778214428265</c:v>
+                  <c:v>389992.51061530097</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.4374397884482208</c:v>
+                  <c:v>393160.78961176169</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.4535996228267836</c:v>
+                  <c:v>394243.07153139927</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.4805458813699364</c:v>
+                  <c:v>393710.54417642875</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.4877646092818484</c:v>
+                  <c:v>401000.88327642059</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.4828050053816089</c:v>
+                  <c:v>400789.03561487945</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5.4872642601914867</c:v>
+                  <c:v>400335.32394307095</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.4957898595804551</c:v>
+                  <c:v>399393.63163614896</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5.4992594494166704</c:v>
+                  <c:v>398381.88710628485</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.4914457426972714</c:v>
+                  <c:v>399724.30291078368</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5.4824619517168323</c:v>
+                  <c:v>401534.10250195052</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>5.4946081391662274</c:v>
+                  <c:v>401046.16396379791</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.5089725408402099</c:v>
+                  <c:v>396481.32851436839</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>5.5129844039304512</c:v>
+                  <c:v>396604.89595966949</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>5.5298305832447596</c:v>
+                  <c:v>399807.14095967996</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5.5613959835338296</c:v>
+                  <c:v>400433.37711545941</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.5708172059581749</c:v>
+                  <c:v>400494.69237654173</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.6507571300202706</c:v>
+                  <c:v>402834.97356046597</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5.6626161908208621</c:v>
+                  <c:v>402471.90373624192</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>5.6698726449388586</c:v>
+                  <c:v>403225.66014035139</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5.6717216144660663</c:v>
+                  <c:v>404241.7529301155</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.7063430523905749</c:v>
+                  <c:v>406428.34253941011</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>5.7314146902155994</c:v>
+                  <c:v>409805.93362261186</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>5.7405016414973176</c:v>
+                  <c:v>411911.79010447086</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>5.761827894107995</c:v>
+                  <c:v>416359.65233785944</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>5.7627130658908703</c:v>
+                  <c:v>422574.28570230992</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>5.7733753523312128</c:v>
+                  <c:v>425395.65964773804</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>5.791639428718411</c:v>
+                  <c:v>431244.59691888973</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>5.8031838885353419</c:v>
+                  <c:v>432435.78011595452</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>5.8067089481055376</c:v>
+                  <c:v>435486.3604382081</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>5.8213176259316048</c:v>
+                  <c:v>437648.56760195253</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>5.8397702022449556</c:v>
+                  <c:v>440763.05950622348</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>5.8470905962575266</c:v>
+                  <c:v>443978.86120116897</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>5.8531583536779692</c:v>
+                  <c:v>442660.63189441146</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>5.8376540824400251</c:v>
+                  <c:v>440470.90768644604</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>5.798850140326774</c:v>
+                  <c:v>432311.66668735462</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>5.7661591867157611</c:v>
+                  <c:v>413003.12550314219</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>5.7774065210041448</c:v>
+                  <c:v>413797.00626406574</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>5.8038065957110518</c:v>
+                  <c:v>416632.07340067555</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>5.8147688358464071</c:v>
+                  <c:v>419763.57001686667</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>5.8185228020031357</c:v>
+                  <c:v>422879.01864168106</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>5.8419773059156173</c:v>
+                  <c:v>430612.28420904285</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>5.8629574231111627</c:v>
+                  <c:v>434462.13854069996</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>5.8713066734521844</c:v>
+                  <c:v>437498.70662731811</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>5.8818711820383518</c:v>
+                  <c:v>444738.77215057274</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>5.8856822982746575</c:v>
+                  <c:v>445744.91614153347</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>5.8931667650262316</c:v>
+                  <c:v>447305.08722162491</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>5.8881806175765918</c:v>
+                  <c:v>446618.60278188973</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>5.9132022318715398</c:v>
+                  <c:v>447439.79189300293</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>5.9022955877226391</c:v>
+                  <c:v>447312.49067172903</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>5.9091943231532511</c:v>
+                  <c:v>448261.96958475857</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>5.8993498529683333</c:v>
+                  <c:v>446988.27576861909</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>5.889673635502251</c:v>
+                  <c:v>444676.66815255891</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>5.9036086590529475</c:v>
+                  <c:v>449149.22690770618</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>5.9140669405302502</c:v>
+                  <c:v>450947.93509937567</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>5.9209191512311126</c:v>
+                  <c:v>451956.56582750776</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>5.9359977113274605</c:v>
+                  <c:v>455831.29602570942</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>5.9387698227831178</c:v>
+                  <c:v>456094.84894104401</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>5.9471007658980959</c:v>
+                  <c:v>458487.32101648307</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>5.9521232982920189</c:v>
+                  <c:v>461142.27300974168</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>5.9594864353699855</c:v>
+                  <c:v>460988.55599470972</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>5.963604157476242</c:v>
+                  <c:v>463445.30863375531</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>5.9742707605807857</c:v>
+                  <c:v>465472.26006543729</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>5.9808543003063503</c:v>
+                  <c:v>467589.59606753167</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>5.9865231750711807</c:v>
+                  <c:v>470824.08140218642</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>5.9873887103345647</c:v>
+                  <c:v>471817.75108486839</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>5.985317325353706</c:v>
+                  <c:v>473627.57607226225</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>5.9898505541668614</c:v>
+                  <c:v>475935.01747389167</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>6.0122908507193467</c:v>
+                  <c:v>481658.4540046716</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>6.0187050745418507</c:v>
+                  <c:v>485314.79423523205</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>6.0188843277252904</c:v>
+                  <c:v>488877.46639867494</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>6.0257354403935492</c:v>
+                  <c:v>493601.10887443885</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>6.0324640309889865</c:v>
+                  <c:v>491814.00661573501</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>6.0322366715132922</c:v>
+                  <c:v>495098.66101571824</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>6.0337630160364073</c:v>
+                  <c:v>492842.84329747915</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>6.0403111307190693</c:v>
+                  <c:v>495237.24465898122</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>6.0382834830584811</c:v>
+                  <c:v>498589.035121897</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>6.0426471670868933</c:v>
+                  <c:v>499330.98937043175</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>6.0447787917426696</c:v>
+                  <c:v>500728.82573688036</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>6.0365007436176228</c:v>
+                  <c:v>499219.00968419871</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>6.0193934024206754</c:v>
+                  <c:v>486612.43347513938</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>5.9148522685650029</c:v>
+                  <c:v>440176.25414027856</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>6.0221478245151809</c:v>
+                  <c:v>482715.93603525637</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>6.0474933229292063</c:v>
+                  <c:v>486132.71388082439</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>6.0383315960257393</c:v>
+                  <c:v>484613.29641875572</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>6.0400704190689112</c:v>
+                  <c:v>495676.15725453012</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>6.0203670842527988</c:v>
+                  <c:v>498631.65235113032</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>6.0301830365597979</c:v>
+                  <c:v>501662.51726277702</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>6.0482020596656749</c:v>
+                  <c:v>504981.40358935756</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>6.0543445055551768</c:v>
+                  <c:v>506241.51152206544</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>6.0724583530570779</c:v>
+                  <c:v>507564.59127744631</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>6.075001013130116</c:v>
+                  <c:v>506140.35099132883</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>6.0752757163689424</c:v>
+                  <c:v>504602.36823800305</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>6.0753513023312991</c:v>
+                  <c:v>505094.71566158708</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>6.0700629995186137</c:v>
+                  <c:v>505591.81632105267</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12554,7 +12554,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C87C-EF4F-B07C-F36CC9F5630D}"/>
+              <c16:uniqueId val="{00000000-46A0-C648-BB5B-B52632777B18}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12567,11 +12567,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="543361680"/>
-        <c:axId val="262638176"/>
+        <c:axId val="515972640"/>
+        <c:axId val="515974352"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="543361680"/>
+        <c:axId val="515972640"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12613,7 +12613,7 @@
             <a:endParaRPr lang="cs-CZ"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="262638176"/>
+        <c:crossAx val="515974352"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12621,7 +12621,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="262638176"/>
+        <c:axId val="515974352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12672,543 +12672,7 @@
             <a:endParaRPr lang="cs-CZ"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="543361680"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="cs-CZ"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="cs-CZ"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="cs-CZ"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>List2!$B$2:$B$96</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="95"/>
-                <c:pt idx="0">
-                  <c:v>265447</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>273804</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>284184</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>302375</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>307443</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>303952</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>307089</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>313177</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>315689</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>310060</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>303712</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>312326</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>322829</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>325825</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>338712</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>364247</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>372235</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>447463</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>459850</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>467598</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>469593</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>508561</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>538784</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>550176</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>577867</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>579046</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>593438</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>618927</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>635600</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>640780</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>662701</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>691465</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>703219</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>713113</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>688104</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>629289</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>583659</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>598972</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>636512</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>652783</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>658450</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>694988</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>729386</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>743544</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>761853</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>768568</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>781928</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>773002</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>818846</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>798538</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>811324</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>793140</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>775664</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>800956</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>820478</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>833526</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>862974</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>868500</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>885321</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>895619</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>910933</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>919611</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>942477</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>956873</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>969445</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>971379</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>966757</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>976901</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>1028705</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>1044011</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>1044442</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>1061049</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>1077616</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>1077052</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>1080844</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>1097264</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>1092153</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>1103182</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>1108610</c:v>
-                </c:pt>
-                <c:pt idx="79">
-                  <c:v>1087679</c:v>
-                </c:pt>
-                <c:pt idx="80">
-                  <c:v>1045667</c:v>
-                </c:pt>
-                <c:pt idx="81">
-                  <c:v>821963</c:v>
-                </c:pt>
-                <c:pt idx="82">
-                  <c:v>1052320</c:v>
-                </c:pt>
-                <c:pt idx="83">
-                  <c:v>1115561</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>1092274</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>1096656</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>1048014</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>1071971</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>1117383</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>1133299</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>1181567</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>1188505</c:v>
-                </c:pt>
-                <c:pt idx="92">
-                  <c:v>1189257</c:v>
-                </c:pt>
-                <c:pt idx="93">
-                  <c:v>1189464</c:v>
-                </c:pt>
-                <c:pt idx="94">
-                  <c:v>1175068</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-CB24-EF43-B722-9B954042BA85}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:smooth val="0"/>
-        <c:axId val="602791504"/>
-        <c:axId val="602405216"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="602791504"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="cs-CZ"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="602405216"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="602405216"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="cs-CZ"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="602791504"/>
+        <c:crossAx val="515972640"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13505,46 +12969,6 @@
 </file>
 
 <file path=xl/charts/colors7.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors8.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -17196,522 +16620,6 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -17937,23 +16845,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>468168</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>6350</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>80818</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>204355</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>81395</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>112568</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>496454</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>38101</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Graf 1">
+        <xdr:cNvPr id="4" name="Graf 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{755AD7B8-D6DB-42FA-801B-FF3EF4BF8656}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{91C7C163-4623-CBAB-0125-73F1320696B6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -17966,42 +16874,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>75177</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>13314</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>519676</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>114915</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Graf 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F66BF95-EE0B-157E-7608-77A2E4F08D67}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -29114,873 +27986,2313 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1338CA2A-5E83-A54D-B63E-F215F1BA064A}">
-  <dimension ref="B1:C96"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.33203125" style="1" customWidth="1"/>
+    <col min="1" max="6" width="11.33203125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B1" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="11" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B2" s="1">
-        <v>265447</v>
-      </c>
-      <c r="C2">
-        <f>LOG10(B2)</f>
-        <v>5.4239778214428265</v>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="5">
+        <v>595801.59999999998</v>
+      </c>
+      <c r="B2" s="5">
+        <v>10570.2</v>
+      </c>
+      <c r="C2" s="5">
+        <v>60209.936173883041</v>
+      </c>
+      <c r="D2" s="5">
+        <v>431559.5</v>
+      </c>
+      <c r="E2" s="5">
+        <v>62060.1</v>
+      </c>
+      <c r="F2" s="5">
+        <v>388892.7</v>
+      </c>
+      <c r="G2">
+        <f>A2*0.518+B2*0.128+C2*0.111+D2*0.086+E2*0.076+F2*0.081</f>
+        <v>389992.51061530097</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B3" s="1">
-        <v>273804</v>
-      </c>
-      <c r="C3">
-        <f t="shared" ref="C3:C66" si="0">LOG10(B3)</f>
-        <v>5.4374397884482208</v>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5">
+        <v>600554.6</v>
+      </c>
+      <c r="B3" s="5">
+        <v>10620.96</v>
+      </c>
+      <c r="C3" s="5">
+        <v>60402.352538393818</v>
+      </c>
+      <c r="D3" s="5">
+        <v>436384.2</v>
+      </c>
+      <c r="E3" s="5">
+        <v>62795.4</v>
+      </c>
+      <c r="F3" s="5">
+        <v>391455.2</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G66" si="0">A3*0.518+B3*0.128+C3*0.111+D3*0.086+E3*0.076+F3*0.081</f>
+        <v>393160.78961176169</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" s="1">
-        <v>284184</v>
-      </c>
-      <c r="C4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="5">
+        <v>600993.30000000005</v>
+      </c>
+      <c r="B4" s="5">
+        <v>10623.35</v>
+      </c>
+      <c r="C4" s="5">
+        <v>62404.981363956889</v>
+      </c>
+      <c r="D4" s="5">
+        <v>439740.2</v>
+      </c>
+      <c r="E4" s="5">
+        <v>63546.9</v>
+      </c>
+      <c r="F4" s="5">
+        <v>394994.8</v>
+      </c>
+      <c r="G4">
         <f t="shared" si="0"/>
-        <v>5.4535996228267836</v>
+        <v>394243.07153139927</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B5" s="1">
-        <v>302375</v>
-      </c>
-      <c r="C5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="5">
+        <v>598434</v>
+      </c>
+      <c r="B5" s="5">
+        <v>10521.37</v>
+      </c>
+      <c r="C5" s="5">
+        <v>64470.388436294917</v>
+      </c>
+      <c r="D5" s="5">
+        <v>442413.8</v>
+      </c>
+      <c r="E5" s="5">
+        <v>64034.3</v>
+      </c>
+      <c r="F5" s="5">
+        <v>398822.1</v>
+      </c>
+      <c r="G5">
         <f t="shared" si="0"/>
-        <v>5.4805458813699364</v>
+        <v>393710.54417642875</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B6" s="1">
-        <v>307443</v>
-      </c>
-      <c r="C6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="5">
+        <v>611139</v>
+      </c>
+      <c r="B6" s="5">
+        <v>10711.84</v>
+      </c>
+      <c r="C6" s="5">
+        <v>66631.591499284536</v>
+      </c>
+      <c r="D6" s="5">
+        <v>444726.2</v>
+      </c>
+      <c r="E6" s="5">
+        <v>63926.6</v>
+      </c>
+      <c r="F6" s="5">
+        <v>401960.3</v>
+      </c>
+      <c r="G6">
         <f t="shared" si="0"/>
-        <v>5.4877646092818484</v>
+        <v>401000.88327642059</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B7" s="1">
-        <v>303952</v>
-      </c>
-      <c r="C7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="5">
+        <v>609603.5</v>
+      </c>
+      <c r="B7" s="5">
+        <v>10841.77</v>
+      </c>
+      <c r="C7" s="5">
+        <v>71963.002296211256</v>
+      </c>
+      <c r="D7" s="5">
+        <v>444833.7</v>
+      </c>
+      <c r="E7" s="5">
+        <v>63763.8</v>
+      </c>
+      <c r="F7" s="5">
+        <v>401691.8</v>
+      </c>
+      <c r="G7">
         <f t="shared" si="0"/>
-        <v>5.4828050053816089</v>
+        <v>400789.03561487945</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B8" s="1">
-        <v>307089</v>
-      </c>
-      <c r="C8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="5">
+        <v>609603.5</v>
+      </c>
+      <c r="B8" s="5">
+        <v>10815.18</v>
+      </c>
+      <c r="C8" s="5">
+        <v>66980.085613251445</v>
+      </c>
+      <c r="D8" s="5">
+        <v>447366.40000000002</v>
+      </c>
+      <c r="E8" s="5">
+        <v>63899.199999999997</v>
+      </c>
+      <c r="F8" s="5">
+        <v>400144.8</v>
+      </c>
+      <c r="G8">
         <f t="shared" si="0"/>
-        <v>5.4872642601914867</v>
+        <v>400335.32394307095</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B9" s="1">
-        <v>313177</v>
-      </c>
-      <c r="C9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="5">
+        <v>607702.4</v>
+      </c>
+      <c r="B9" s="5">
+        <v>11161.12</v>
+      </c>
+      <c r="C9" s="5">
+        <v>68739.589875215024</v>
+      </c>
+      <c r="D9" s="5">
+        <v>445422.5</v>
+      </c>
+      <c r="E9" s="5">
+        <v>64129.7</v>
+      </c>
+      <c r="F9" s="5">
+        <v>399566.4</v>
+      </c>
+      <c r="G9">
         <f t="shared" si="0"/>
-        <v>5.4957898595804551</v>
+        <v>399393.63163614896</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B10" s="1">
-        <v>315689</v>
-      </c>
-      <c r="C10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="5">
+        <v>604868.80000000005</v>
+      </c>
+      <c r="B10" s="5">
+        <v>11136</v>
+      </c>
+      <c r="C10" s="5">
+        <v>70018.462218782821</v>
+      </c>
+      <c r="D10" s="5">
+        <v>447992.4</v>
+      </c>
+      <c r="E10" s="5">
+        <v>64865.1</v>
+      </c>
+      <c r="F10" s="5">
+        <v>400065.4</v>
+      </c>
+      <c r="G10">
         <f t="shared" si="0"/>
-        <v>5.4992594494166704</v>
+        <v>398381.88710628485</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B11" s="1">
-        <v>310060</v>
-      </c>
-      <c r="C11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="5">
+        <v>607208.69999999995</v>
+      </c>
+      <c r="B11" s="5">
+        <v>11227.11</v>
+      </c>
+      <c r="C11" s="5">
+        <v>68612.957034087551</v>
+      </c>
+      <c r="D11" s="5">
+        <v>450086.7</v>
+      </c>
+      <c r="E11" s="5">
+        <v>64930.9</v>
+      </c>
+      <c r="F11" s="5">
+        <v>401171.4</v>
+      </c>
+      <c r="G11">
         <f t="shared" si="0"/>
-        <v>5.4914457426972714</v>
+        <v>399724.30291078368</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B12" s="1">
-        <v>303712</v>
-      </c>
-      <c r="C12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="5">
+        <v>611376.69999999995</v>
+      </c>
+      <c r="B12" s="5">
+        <v>11560.12</v>
+      </c>
+      <c r="C12" s="5">
+        <v>63086.890468022539</v>
+      </c>
+      <c r="D12" s="5">
+        <v>451943.5</v>
+      </c>
+      <c r="E12" s="5">
+        <v>64999.1</v>
+      </c>
+      <c r="F12" s="5">
+        <v>401871.1</v>
+      </c>
+      <c r="G12">
         <f t="shared" si="0"/>
-        <v>5.4824619517168323</v>
+        <v>401534.10250195052</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B13" s="1">
-        <v>312326</v>
-      </c>
-      <c r="C13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="5">
+        <v>609694.9</v>
+      </c>
+      <c r="B13" s="5">
+        <v>11562.5</v>
+      </c>
+      <c r="C13" s="5">
+        <v>64737.703277458095</v>
+      </c>
+      <c r="D13" s="5">
+        <v>452336</v>
+      </c>
+      <c r="E13" s="5">
+        <v>64706.400000000001</v>
+      </c>
+      <c r="F13" s="5">
+        <v>404194.3</v>
+      </c>
+      <c r="G13">
         <f t="shared" si="0"/>
-        <v>5.4946081391662274</v>
+        <v>401046.16396379791</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B14" s="1">
-        <v>322829</v>
-      </c>
-      <c r="C14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="5">
+        <v>601413.9</v>
+      </c>
+      <c r="B14" s="5">
+        <v>11749.97</v>
+      </c>
+      <c r="C14" s="5">
+        <v>62028.668958273665</v>
+      </c>
+      <c r="D14" s="5">
+        <v>453740.2</v>
+      </c>
+      <c r="E14" s="5">
+        <v>64937</v>
+      </c>
+      <c r="F14" s="5">
+        <v>402504.7</v>
+      </c>
+      <c r="G14">
         <f t="shared" si="0"/>
-        <v>5.5089725408402099</v>
+        <v>396481.32851436839</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B15" s="1">
-        <v>325825</v>
-      </c>
-      <c r="C15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="5">
+        <v>602291.30000000005</v>
+      </c>
+      <c r="B15" s="5">
+        <v>11923.64</v>
+      </c>
+      <c r="C15" s="5">
+        <v>60648.20936639118</v>
+      </c>
+      <c r="D15" s="5">
+        <v>451715.5</v>
+      </c>
+      <c r="E15" s="5">
+        <v>65353.7</v>
+      </c>
+      <c r="F15" s="5">
+        <v>401795.2</v>
+      </c>
+      <c r="G15">
         <f t="shared" si="0"/>
-        <v>5.5129844039304512</v>
+        <v>396604.89595966949</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B16" s="1">
-        <v>338712</v>
-      </c>
-      <c r="C16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="5">
+        <v>607775.30000000005</v>
+      </c>
+      <c r="B16" s="5">
+        <v>11896.79</v>
+      </c>
+      <c r="C16" s="5">
+        <v>60481.127384504114</v>
+      </c>
+      <c r="D16" s="5">
+        <v>456584</v>
+      </c>
+      <c r="E16" s="5">
+        <v>65939.5</v>
+      </c>
+      <c r="F16" s="5">
+        <v>400811.3</v>
+      </c>
+      <c r="G16">
         <f t="shared" si="0"/>
-        <v>5.5298305832447596</v>
+        <v>399807.14095967996</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B17" s="1">
-        <v>364247</v>
-      </c>
-      <c r="C17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="5">
+        <v>608506.6</v>
+      </c>
+      <c r="B17" s="5">
+        <v>12145.77</v>
+      </c>
+      <c r="C17" s="5">
+        <v>58332.302301436241</v>
+      </c>
+      <c r="D17" s="5">
+        <v>458175.6</v>
+      </c>
+      <c r="E17" s="5">
+        <v>66098.399999999994</v>
+      </c>
+      <c r="F17" s="5">
+        <v>404578.2</v>
+      </c>
+      <c r="G17">
         <f t="shared" si="0"/>
-        <v>5.5613959835338296</v>
+        <v>400433.37711545941</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="1">
-        <v>372235</v>
-      </c>
-      <c r="C18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="5">
+        <v>607574.30000000005</v>
+      </c>
+      <c r="B18" s="5">
+        <v>12338.54</v>
+      </c>
+      <c r="C18" s="5">
+        <v>57798.232941816888</v>
+      </c>
+      <c r="D18" s="5">
+        <v>463165.2</v>
+      </c>
+      <c r="E18" s="5">
+        <v>66267.8</v>
+      </c>
+      <c r="F18" s="5">
+        <v>406268</v>
+      </c>
+      <c r="G18">
         <f t="shared" si="0"/>
-        <v>5.5708172059581749</v>
+        <v>400494.69237654173</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B19" s="1">
-        <v>447463</v>
-      </c>
-      <c r="C19">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="5">
+        <v>611157.30000000005</v>
+      </c>
+      <c r="B19" s="5">
+        <v>12325.91</v>
+      </c>
+      <c r="C19" s="5">
+        <v>59381.658382575675</v>
+      </c>
+      <c r="D19" s="5">
+        <v>465196.1</v>
+      </c>
+      <c r="E19" s="5">
+        <v>66940.600000000006</v>
+      </c>
+      <c r="F19" s="5">
+        <v>407309.4</v>
+      </c>
+      <c r="G19">
         <f t="shared" si="0"/>
-        <v>5.6507571300202706</v>
+        <v>402834.97356046597</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B20" s="1">
-        <v>459850</v>
-      </c>
-      <c r="C20">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="5">
+        <v>609183</v>
+      </c>
+      <c r="B20" s="5">
+        <v>12711.9</v>
+      </c>
+      <c r="C20" s="5">
+        <v>62893.503029206979</v>
+      </c>
+      <c r="D20" s="5">
+        <v>466821.4</v>
+      </c>
+      <c r="E20" s="5">
+        <v>67693.7</v>
+      </c>
+      <c r="F20" s="5">
+        <v>407598.1</v>
+      </c>
+      <c r="G20">
         <f t="shared" si="0"/>
-        <v>5.6626161908208621</v>
+        <v>402471.90373624192</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B21" s="1">
-        <v>467598</v>
-      </c>
-      <c r="C21">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="5">
+        <v>608963.69999999995</v>
+      </c>
+      <c r="B21" s="5">
+        <v>12899.91</v>
+      </c>
+      <c r="C21" s="5">
+        <v>66348.660904066885</v>
+      </c>
+      <c r="D21" s="5">
+        <v>470976.1</v>
+      </c>
+      <c r="E21" s="5">
+        <v>67926</v>
+      </c>
+      <c r="F21" s="5">
+        <v>408645.1</v>
+      </c>
+      <c r="G21">
         <f t="shared" si="0"/>
-        <v>5.6698726449388586</v>
+        <v>403225.66014035139</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B22" s="1">
-        <v>469593</v>
-      </c>
-      <c r="C22">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="5">
+        <v>609932.4</v>
+      </c>
+      <c r="B22" s="5">
+        <v>12993.91</v>
+      </c>
+      <c r="C22" s="5">
+        <v>70154.468919959269</v>
+      </c>
+      <c r="D22" s="5">
+        <v>472409.7</v>
+      </c>
+      <c r="E22" s="5">
+        <v>68143.8</v>
+      </c>
+      <c r="F22" s="5">
+        <v>407904.2</v>
+      </c>
+      <c r="G22">
         <f t="shared" si="0"/>
-        <v>5.6717216144660663</v>
+        <v>404241.7529301155</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B23" s="1">
-        <v>508561</v>
-      </c>
-      <c r="C23">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="5">
+        <v>613588.6</v>
+      </c>
+      <c r="B23" s="5">
+        <v>13323.16</v>
+      </c>
+      <c r="C23" s="5">
+        <v>68714.922156848508</v>
+      </c>
+      <c r="D23" s="5">
+        <v>473457.4</v>
+      </c>
+      <c r="E23" s="5">
+        <v>68607.899999999994</v>
+      </c>
+      <c r="F23" s="5">
+        <v>411422.1</v>
+      </c>
+      <c r="G23">
         <f t="shared" si="0"/>
-        <v>5.7063430523905749</v>
+        <v>406428.34253941011</v>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B24" s="1">
-        <v>538784</v>
-      </c>
-      <c r="C24">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="5">
+        <v>618414.80000000005</v>
+      </c>
+      <c r="B24" s="5">
+        <v>13541.41</v>
+      </c>
+      <c r="C24" s="5">
+        <v>71893.843627133814</v>
+      </c>
+      <c r="D24" s="5">
+        <v>477015.1</v>
+      </c>
+      <c r="E24" s="5">
+        <v>68789.2</v>
+      </c>
+      <c r="F24" s="5">
+        <v>413608.3</v>
+      </c>
+      <c r="G24">
         <f t="shared" si="0"/>
-        <v>5.7314146902155994</v>
+        <v>409805.93362261186</v>
       </c>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B25" s="1">
-        <v>550176</v>
-      </c>
-      <c r="C25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="5">
+        <v>620754.80000000005</v>
+      </c>
+      <c r="B25" s="5">
+        <v>13682.74</v>
+      </c>
+      <c r="C25" s="5">
+        <v>75119.968328565592</v>
+      </c>
+      <c r="D25" s="5">
+        <v>480313.8</v>
+      </c>
+      <c r="E25" s="5">
+        <v>69810.8</v>
+      </c>
+      <c r="F25" s="5">
+        <v>415536.9</v>
+      </c>
+      <c r="G25">
         <f t="shared" si="0"/>
-        <v>5.7405016414973176</v>
+        <v>411911.79010447086</v>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B26" s="1">
-        <v>577867</v>
-      </c>
-      <c r="C26">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="5">
+        <v>627683</v>
+      </c>
+      <c r="B26" s="5">
+        <v>14075.22</v>
+      </c>
+      <c r="C26" s="5">
+        <v>77897.35565639181</v>
+      </c>
+      <c r="D26" s="5">
+        <v>484537.1</v>
+      </c>
+      <c r="E26" s="5">
+        <v>70459.600000000006</v>
+      </c>
+      <c r="F26" s="5">
+        <v>416623.5</v>
+      </c>
+      <c r="G26">
         <f t="shared" si="0"/>
-        <v>5.761827894107995</v>
+        <v>416359.65233785944</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B27" s="1">
-        <v>579046</v>
-      </c>
-      <c r="C27">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="5">
+        <v>638432</v>
+      </c>
+      <c r="B27" s="5">
+        <v>14451.5</v>
+      </c>
+      <c r="C27" s="5">
+        <v>77413.859480269501</v>
+      </c>
+      <c r="D27" s="5">
+        <v>490358.6</v>
+      </c>
+      <c r="E27" s="5">
+        <v>70810.3</v>
+      </c>
+      <c r="F27" s="5">
+        <v>418164.9</v>
+      </c>
+      <c r="G27">
         <f t="shared" si="0"/>
-        <v>5.7627130658908703</v>
+        <v>422574.28570230992</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B28" s="1">
-        <v>593438</v>
-      </c>
-      <c r="C28">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="5">
+        <v>643258.1</v>
+      </c>
+      <c r="B28" s="5">
+        <v>14654.97</v>
+      </c>
+      <c r="C28" s="5">
+        <v>78566.760249892512</v>
+      </c>
+      <c r="D28" s="5">
+        <v>490693.3</v>
+      </c>
+      <c r="E28" s="5">
+        <v>71231.899999999994</v>
+      </c>
+      <c r="F28" s="5">
+        <v>419481.1</v>
+      </c>
+      <c r="G28">
         <f t="shared" si="0"/>
-        <v>5.7733753523312128</v>
+        <v>425395.65964773804</v>
       </c>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B29" s="1">
-        <v>618927</v>
-      </c>
-      <c r="C29">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="5">
+        <v>652690.9</v>
+      </c>
+      <c r="B29" s="5">
+        <v>15108.56</v>
+      </c>
+      <c r="C29" s="5">
+        <v>79614.740890898698</v>
+      </c>
+      <c r="D29" s="5">
+        <v>493373.9</v>
+      </c>
+      <c r="E29" s="5">
+        <v>72254.3</v>
+      </c>
+      <c r="F29" s="5">
+        <v>425408.6</v>
+      </c>
+      <c r="G29">
         <f t="shared" si="0"/>
-        <v>5.791639428718411</v>
+        <v>431244.59691888973</v>
       </c>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B30" s="1">
-        <v>635600</v>
-      </c>
-      <c r="C30">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="5">
+        <v>653550.19999999995</v>
+      </c>
+      <c r="B30" s="5">
+        <v>15399.31</v>
+      </c>
+      <c r="C30" s="5">
+        <v>82074.801224815383</v>
+      </c>
+      <c r="D30" s="5">
+        <v>498529.2</v>
+      </c>
+      <c r="E30" s="5">
+        <v>73101.399999999994</v>
+      </c>
+      <c r="F30" s="5">
+        <v>424520.3</v>
+      </c>
+      <c r="G30">
         <f t="shared" si="0"/>
-        <v>5.8031838885353419</v>
+        <v>432435.78011595452</v>
       </c>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B31" s="1">
-        <v>640780</v>
-      </c>
-      <c r="C31">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="5">
+        <v>657864.4</v>
+      </c>
+      <c r="B31" s="5">
+        <v>15808.24</v>
+      </c>
+      <c r="C31" s="5">
+        <v>85024.338902775955</v>
+      </c>
+      <c r="D31" s="5">
+        <v>501805.9</v>
+      </c>
+      <c r="E31" s="5">
+        <v>73822.7</v>
+      </c>
+      <c r="F31" s="5">
+        <v>425748.3</v>
+      </c>
+      <c r="G31">
         <f t="shared" si="0"/>
-        <v>5.8067089481055376</v>
+        <v>435486.3604382081</v>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B32" s="1">
-        <v>662701</v>
-      </c>
-      <c r="C32">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="5">
+        <v>661227.9</v>
+      </c>
+      <c r="B32" s="5">
+        <v>16213.17</v>
+      </c>
+      <c r="C32" s="5">
+        <v>86751.873350923473</v>
+      </c>
+      <c r="D32" s="5">
+        <v>503386</v>
+      </c>
+      <c r="E32" s="5">
+        <v>74202.8</v>
+      </c>
+      <c r="F32" s="5">
+        <v>425890.9</v>
+      </c>
+      <c r="G32">
         <f t="shared" si="0"/>
-        <v>5.8213176259316048</v>
+        <v>437648.56760195253</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B33" s="1">
-        <v>691465</v>
-      </c>
-      <c r="C33">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="5">
+        <v>666127</v>
+      </c>
+      <c r="B33" s="5">
+        <v>17157.490000000002</v>
+      </c>
+      <c r="C33" s="5">
+        <v>91108.162038049413</v>
+      </c>
+      <c r="D33" s="5">
+        <v>503917.9</v>
+      </c>
+      <c r="E33" s="5">
+        <v>74193.899999999994</v>
+      </c>
+      <c r="F33" s="5">
+        <v>424993</v>
+      </c>
+      <c r="G33">
         <f t="shared" si="0"/>
-        <v>5.8397702022449556</v>
+        <v>440763.05950622348</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B34" s="1">
-        <v>703219</v>
-      </c>
-      <c r="C34">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="5">
+        <v>670039.30000000005</v>
+      </c>
+      <c r="B34" s="5">
+        <v>16737.7</v>
+      </c>
+      <c r="C34" s="5">
+        <v>94687.29550602645</v>
+      </c>
+      <c r="D34" s="5">
+        <v>508276.5</v>
+      </c>
+      <c r="E34" s="5">
+        <v>75743.600000000006</v>
+      </c>
+      <c r="F34" s="5">
+        <v>429351.8</v>
+      </c>
+      <c r="G34">
         <f t="shared" si="0"/>
-        <v>5.8470905962575266</v>
+        <v>443978.86120116897</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B35" s="1">
-        <v>713113</v>
-      </c>
-      <c r="C35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="5">
+        <v>667626.30000000005</v>
+      </c>
+      <c r="B35" s="5">
+        <v>16905.61</v>
+      </c>
+      <c r="C35" s="5">
+        <v>99926.474904608156</v>
+      </c>
+      <c r="D35" s="5">
+        <v>504490.8</v>
+      </c>
+      <c r="E35" s="5">
+        <v>75471.8</v>
+      </c>
+      <c r="F35" s="5">
+        <v>425338.1</v>
+      </c>
+      <c r="G35">
         <f t="shared" si="0"/>
-        <v>5.8531583536779692</v>
+        <v>442660.63189441146</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B36" s="1">
-        <v>688104</v>
-      </c>
-      <c r="C36">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="5">
+        <v>663970</v>
+      </c>
+      <c r="B36" s="5">
+        <v>17161.54</v>
+      </c>
+      <c r="C36" s="5">
+        <v>102876.66636437834</v>
+      </c>
+      <c r="D36" s="5">
+        <v>503262.8</v>
+      </c>
+      <c r="E36" s="5">
+        <v>74973.7</v>
+      </c>
+      <c r="F36" s="5">
+        <v>419010.6</v>
+      </c>
+      <c r="G36">
         <f t="shared" si="0"/>
-        <v>5.8376540824400251</v>
+        <v>440470.90768644604</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B37" s="1">
-        <v>629289</v>
-      </c>
-      <c r="C37">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="5">
+        <v>653659.5</v>
+      </c>
+      <c r="B37" s="5">
+        <v>17288.75</v>
+      </c>
+      <c r="C37" s="5">
+        <v>90531.971958149661</v>
+      </c>
+      <c r="D37" s="5">
+        <v>496876.79999999999</v>
+      </c>
+      <c r="E37" s="5">
+        <v>73180.5</v>
+      </c>
+      <c r="F37" s="5">
+        <v>409394</v>
+      </c>
+      <c r="G37">
         <f t="shared" si="0"/>
-        <v>5.798850140326774</v>
+        <v>432311.66668735462</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B38" s="1">
-        <v>583659</v>
-      </c>
-      <c r="C38">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="5">
+        <v>623021.30000000005</v>
+      </c>
+      <c r="B38" s="5">
+        <v>15712.19</v>
+      </c>
+      <c r="C38" s="5">
+        <v>76677.358406686224</v>
+      </c>
+      <c r="D38" s="5">
+        <v>487419.9</v>
+      </c>
+      <c r="E38" s="5">
+        <v>72208.600000000006</v>
+      </c>
+      <c r="F38" s="5">
+        <v>399380</v>
+      </c>
+      <c r="G38">
         <f t="shared" si="0"/>
-        <v>5.7661591867157611</v>
+        <v>413003.12550314219</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B39" s="1">
-        <v>598972</v>
-      </c>
-      <c r="C39">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="5">
+        <v>624556.9</v>
+      </c>
+      <c r="B39" s="5">
+        <v>15932.8</v>
+      </c>
+      <c r="C39" s="5">
+        <v>77654.425802394268</v>
+      </c>
+      <c r="D39" s="5">
+        <v>488279.7</v>
+      </c>
+      <c r="E39" s="5">
+        <v>71905.600000000006</v>
+      </c>
+      <c r="F39" s="5">
+        <v>397044.6</v>
+      </c>
+      <c r="G39">
         <f t="shared" si="0"/>
-        <v>5.7774065210041448</v>
+        <v>413797.00626406574</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B40" s="1">
-        <v>636512</v>
-      </c>
-      <c r="C40">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="5">
+        <v>628432.6</v>
+      </c>
+      <c r="B40" s="5">
+        <v>16183.84</v>
+      </c>
+      <c r="C40" s="5">
+        <v>82991.805231311635</v>
+      </c>
+      <c r="D40" s="5">
+        <v>489379.3</v>
+      </c>
+      <c r="E40" s="5">
+        <v>72271.399999999994</v>
+      </c>
+      <c r="F40" s="5">
+        <v>398038.5</v>
+      </c>
+      <c r="G40">
         <f t="shared" si="0"/>
-        <v>5.8038065957110518</v>
+        <v>416632.07340067555</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B41" s="1">
-        <v>652783</v>
-      </c>
-      <c r="C41">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="5">
+        <v>633258.80000000005</v>
+      </c>
+      <c r="B41" s="5">
+        <v>16496.259999999998</v>
+      </c>
+      <c r="C41" s="5">
+        <v>84885.926458258473</v>
+      </c>
+      <c r="D41" s="5">
+        <v>492862.2</v>
+      </c>
+      <c r="E41" s="5">
+        <v>72288.2</v>
+      </c>
+      <c r="F41" s="5">
+        <v>399032.1</v>
+      </c>
+      <c r="G41">
         <f t="shared" si="0"/>
-        <v>5.8147688358464071</v>
+        <v>419763.57001686667</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B42" s="1">
-        <v>658450</v>
-      </c>
-      <c r="C42">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="5">
+        <v>637864.9</v>
+      </c>
+      <c r="B42" s="5">
+        <v>16907.79</v>
+      </c>
+      <c r="C42" s="5">
+        <v>88559.030825955007</v>
+      </c>
+      <c r="D42" s="5">
+        <v>494372.5</v>
+      </c>
+      <c r="E42" s="5">
+        <v>72116.899999999994</v>
+      </c>
+      <c r="F42" s="5">
+        <v>400911.5</v>
+      </c>
+      <c r="G42">
         <f t="shared" si="0"/>
-        <v>5.8185228020031357</v>
+        <v>422879.01864168106</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B43" s="1">
-        <v>694988</v>
-      </c>
-      <c r="C43">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="5">
+        <v>651685.4</v>
+      </c>
+      <c r="B43" s="5">
+        <v>17066.22</v>
+      </c>
+      <c r="C43" s="5">
+        <v>89201.413955340919</v>
+      </c>
+      <c r="D43" s="5">
+        <v>496683.1</v>
+      </c>
+      <c r="E43" s="5">
+        <v>73118.5</v>
+      </c>
+      <c r="F43" s="5">
+        <v>403477.3</v>
+      </c>
+      <c r="G43">
         <f t="shared" si="0"/>
-        <v>5.8419773059156173</v>
+        <v>430612.28420904285</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B44" s="1">
-        <v>729386</v>
-      </c>
-      <c r="C44">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="5">
+        <v>657974.1</v>
+      </c>
+      <c r="B44" s="5">
+        <v>17272.09</v>
+      </c>
+      <c r="C44" s="5">
+        <v>90438.870456756544</v>
+      </c>
+      <c r="D44" s="5">
+        <v>499935.8</v>
+      </c>
+      <c r="E44" s="5">
+        <v>73914.600000000006</v>
+      </c>
+      <c r="F44" s="5">
+        <v>404568.2</v>
+      </c>
+      <c r="G44">
         <f t="shared" si="0"/>
-        <v>5.8629574231111627</v>
+        <v>434462.13854069996</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B45" s="1">
-        <v>743544</v>
-      </c>
-      <c r="C45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="5">
+        <v>662288.5</v>
+      </c>
+      <c r="B45" s="5">
+        <v>17403.099999999999</v>
+      </c>
+      <c r="C45" s="5">
+        <v>92156.985831694648</v>
+      </c>
+      <c r="D45" s="5">
+        <v>502940.7</v>
+      </c>
+      <c r="E45" s="5">
+        <v>74564.7</v>
+      </c>
+      <c r="F45" s="5">
+        <v>408104</v>
+      </c>
+      <c r="G45">
         <f t="shared" si="0"/>
-        <v>5.8713066734521844</v>
+        <v>437498.70662731811</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B46" s="1">
-        <v>761853</v>
-      </c>
-      <c r="C46">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="5">
+        <v>674262</v>
+      </c>
+      <c r="B46" s="5">
+        <v>17402.52</v>
+      </c>
+      <c r="C46" s="5">
+        <v>94303.497212366943</v>
+      </c>
+      <c r="D46" s="5">
+        <v>509556.3</v>
+      </c>
+      <c r="E46" s="5">
+        <v>75410.600000000006</v>
+      </c>
+      <c r="F46" s="5">
+        <v>410158</v>
+      </c>
+      <c r="G46">
         <f t="shared" si="0"/>
-        <v>5.8818711820383518</v>
+        <v>444738.77215057274</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B47" s="1">
-        <v>768568</v>
-      </c>
-      <c r="C47">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="5">
+        <v>676090.1</v>
+      </c>
+      <c r="B47" s="5">
+        <v>17564.27</v>
+      </c>
+      <c r="C47" s="5">
+        <v>95167.542175977374</v>
+      </c>
+      <c r="D47" s="5">
+        <v>509632.9</v>
+      </c>
+      <c r="E47" s="5">
+        <v>75392.399999999994</v>
+      </c>
+      <c r="F47" s="5">
+        <v>409384.8</v>
+      </c>
+      <c r="G47">
         <f t="shared" si="0"/>
-        <v>5.8856822982746575</v>
+        <v>445744.91614153347</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B48" s="1">
-        <v>781928</v>
-      </c>
-      <c r="C48">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="5">
+        <v>679746.2</v>
+      </c>
+      <c r="B48" s="5">
+        <v>17642.57</v>
+      </c>
+      <c r="C48" s="5">
+        <v>91803.93478941411</v>
+      </c>
+      <c r="D48" s="5">
+        <v>511235.7</v>
+      </c>
+      <c r="E48" s="5">
+        <v>75841.100000000006</v>
+      </c>
+      <c r="F48" s="5">
+        <v>407628.1</v>
+      </c>
+      <c r="G48">
         <f t="shared" si="0"/>
-        <v>5.8931667650262316</v>
+        <v>447305.08722162491</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B49" s="1">
-        <v>773002</v>
-      </c>
-      <c r="C49">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="5">
+        <v>679673.1</v>
+      </c>
+      <c r="B49" s="5">
+        <v>17841.3</v>
+      </c>
+      <c r="C49" s="5">
+        <v>87037.889926934658</v>
+      </c>
+      <c r="D49" s="5">
+        <v>513035.7</v>
+      </c>
+      <c r="E49" s="5">
+        <v>76058.899999999994</v>
+      </c>
+      <c r="F49" s="5">
+        <v>403722.2</v>
+      </c>
+      <c r="G49">
         <f t="shared" si="0"/>
-        <v>5.8881806175765918</v>
+        <v>446618.60278188973</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B50" s="1">
-        <v>818846</v>
-      </c>
-      <c r="C50">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="5">
+        <v>681117.2</v>
+      </c>
+      <c r="B50" s="5">
+        <v>17864.259999999998</v>
+      </c>
+      <c r="C50" s="5">
+        <v>91093.174891918068</v>
+      </c>
+      <c r="D50" s="5">
+        <v>512791.9</v>
+      </c>
+      <c r="E50" s="5">
+        <v>76249.2</v>
+      </c>
+      <c r="F50" s="5">
+        <v>399112</v>
+      </c>
+      <c r="G50">
         <f t="shared" si="0"/>
-        <v>5.9132022318715398</v>
+        <v>447439.79189300293</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B51" s="1">
-        <v>798538</v>
-      </c>
-      <c r="C51">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="5">
+        <v>681848.5</v>
+      </c>
+      <c r="B51" s="5">
+        <v>17906.580000000002</v>
+      </c>
+      <c r="C51" s="5">
+        <v>90323.840826388085</v>
+      </c>
+      <c r="D51" s="5">
+        <v>510778.2</v>
+      </c>
+      <c r="E51" s="5">
+        <v>76146</v>
+      </c>
+      <c r="F51" s="5">
+        <v>396085.9</v>
+      </c>
+      <c r="G51">
         <f t="shared" si="0"/>
-        <v>5.9022955877226391</v>
+        <v>447312.49067172903</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B52" s="1">
-        <v>811324</v>
-      </c>
-      <c r="C52">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" s="5">
+        <v>683237.7</v>
+      </c>
+      <c r="B52" s="5">
+        <v>17936.939999999999</v>
+      </c>
+      <c r="C52" s="5">
+        <v>93052.506889716198</v>
+      </c>
+      <c r="D52" s="5">
+        <v>512318.2</v>
+      </c>
+      <c r="E52" s="5">
+        <v>76302.8</v>
+      </c>
+      <c r="F52" s="5">
+        <v>393354.4</v>
+      </c>
+      <c r="G52">
         <f t="shared" si="0"/>
-        <v>5.9091943231532511</v>
+        <v>448261.96958475857</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B53" s="1">
-        <v>793140</v>
-      </c>
-      <c r="C53">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="5">
+        <v>681190.40000000002</v>
+      </c>
+      <c r="B53" s="5">
+        <v>17908.43</v>
+      </c>
+      <c r="C53" s="5">
+        <v>93503.781338910092</v>
+      </c>
+      <c r="D53" s="5">
+        <v>512263.5</v>
+      </c>
+      <c r="E53" s="5">
+        <v>75912.2</v>
+      </c>
+      <c r="F53" s="5">
+        <v>390573.6</v>
+      </c>
+      <c r="G53">
         <f t="shared" si="0"/>
-        <v>5.8993498529683333</v>
+        <v>446988.27576861909</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B54" s="1">
-        <v>775664</v>
-      </c>
-      <c r="C54">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="5">
+        <v>677424.3</v>
+      </c>
+      <c r="B54" s="5">
+        <v>17899.41</v>
+      </c>
+      <c r="C54" s="5">
+        <v>92271.115068097599</v>
+      </c>
+      <c r="D54" s="5">
+        <v>513222.9</v>
+      </c>
+      <c r="E54" s="5">
+        <v>75659.199999999997</v>
+      </c>
+      <c r="F54" s="5">
+        <v>387041.9</v>
+      </c>
+      <c r="G54">
         <f t="shared" si="0"/>
-        <v>5.889673635502251</v>
+        <v>444676.66815255891</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B55" s="1">
-        <v>800956</v>
-      </c>
-      <c r="C55">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="5">
+        <v>685321.8</v>
+      </c>
+      <c r="B55" s="5">
+        <v>17978.22</v>
+      </c>
+      <c r="C55" s="5">
+        <v>92030.131961316758</v>
+      </c>
+      <c r="D55" s="5">
+        <v>517731.1</v>
+      </c>
+      <c r="E55" s="5">
+        <v>75821.399999999994</v>
+      </c>
+      <c r="F55" s="5">
+        <v>387020.7</v>
+      </c>
+      <c r="G55">
         <f t="shared" si="0"/>
-        <v>5.9036086590529475</v>
+        <v>449149.22690770618</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B56" s="1">
-        <v>820478</v>
-      </c>
-      <c r="C56">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="5">
+        <v>688831.7</v>
+      </c>
+      <c r="B56" s="5">
+        <v>18078.830000000002</v>
+      </c>
+      <c r="C56" s="5">
+        <v>91624.078913294245</v>
+      </c>
+      <c r="D56" s="5">
+        <v>516499.8</v>
+      </c>
+      <c r="E56" s="5">
+        <v>76041.600000000006</v>
+      </c>
+      <c r="F56" s="5">
+        <v>388279.1</v>
+      </c>
+      <c r="G56">
         <f t="shared" si="0"/>
-        <v>5.9140669405302502</v>
+        <v>450947.93509937567</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B57" s="1">
-        <v>833526</v>
-      </c>
-      <c r="C57">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" s="5">
+        <v>689855.5</v>
+      </c>
+      <c r="B57" s="5">
+        <v>18184.72</v>
+      </c>
+      <c r="C57" s="5">
+        <v>93510.524932501852</v>
+      </c>
+      <c r="D57" s="5">
+        <v>519651.8</v>
+      </c>
+      <c r="E57" s="5">
+        <v>76178.7</v>
+      </c>
+      <c r="F57" s="5">
+        <v>387956.4</v>
+      </c>
+      <c r="G57">
         <f t="shared" si="0"/>
-        <v>5.9209191512311126</v>
+        <v>451956.56582750776</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B58" s="1">
-        <v>862974</v>
-      </c>
-      <c r="C58">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" s="5">
+        <v>697058</v>
+      </c>
+      <c r="B58" s="5">
+        <v>18313.29</v>
+      </c>
+      <c r="C58" s="5">
+        <v>94783.763114499438</v>
+      </c>
+      <c r="D58" s="5">
+        <v>519669.4</v>
+      </c>
+      <c r="E58" s="5">
+        <v>76156.399999999994</v>
+      </c>
+      <c r="F58" s="5">
+        <v>387786.4</v>
+      </c>
+      <c r="G58">
         <f t="shared" si="0"/>
-        <v>5.9359977113274605</v>
+        <v>455831.29602570942</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B59" s="1">
-        <v>868500</v>
-      </c>
-      <c r="C59">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" s="5">
+        <v>696911.7</v>
+      </c>
+      <c r="B59" s="5">
+        <v>18434.48</v>
+      </c>
+      <c r="C59" s="5">
+        <v>96267.802712108474</v>
+      </c>
+      <c r="D59" s="5">
+        <v>520972.4</v>
+      </c>
+      <c r="E59" s="5">
+        <v>76575.8</v>
+      </c>
+      <c r="F59" s="5">
+        <v>387973.6</v>
+      </c>
+      <c r="G59">
         <f t="shared" si="0"/>
-        <v>5.9387698227831178</v>
+        <v>456094.84894104401</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B60" s="1">
-        <v>885321</v>
-      </c>
-      <c r="C60">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" s="5">
+        <v>700787.1</v>
+      </c>
+      <c r="B60" s="5">
+        <v>18589.669999999998</v>
+      </c>
+      <c r="C60" s="5">
+        <v>96858.432941289211</v>
+      </c>
+      <c r="D60" s="5">
+        <v>524292.4</v>
+      </c>
+      <c r="E60" s="5">
+        <v>76671.199999999997</v>
+      </c>
+      <c r="F60" s="5">
+        <v>388057.8</v>
+      </c>
+      <c r="G60">
         <f t="shared" si="0"/>
-        <v>5.9471007658980959</v>
+        <v>458487.32101648307</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B61" s="1">
-        <v>895619</v>
-      </c>
-      <c r="C61">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" s="5">
+        <v>706124.9</v>
+      </c>
+      <c r="B61" s="5">
+        <v>18728.240000000002</v>
+      </c>
+      <c r="C61" s="5">
+        <v>96837.148556230997</v>
+      </c>
+      <c r="D61" s="5">
+        <v>522861.6</v>
+      </c>
+      <c r="E61" s="5">
+        <v>77069.100000000006</v>
+      </c>
+      <c r="F61" s="5">
+        <v>387655.4</v>
+      </c>
+      <c r="G61">
         <f t="shared" si="0"/>
-        <v>5.9521232982920189</v>
+        <v>461142.27300974168</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B62" s="1">
-        <v>910933</v>
-      </c>
-      <c r="C62">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" s="5">
+        <v>704589.7</v>
+      </c>
+      <c r="B62" s="5">
+        <v>19150.150000000001</v>
+      </c>
+      <c r="C62" s="5">
+        <v>98857.606258646207</v>
+      </c>
+      <c r="D62" s="5">
+        <v>525883.5</v>
+      </c>
+      <c r="E62" s="5">
+        <v>76978</v>
+      </c>
+      <c r="F62" s="5">
+        <v>389016.9</v>
+      </c>
+      <c r="G62">
         <f t="shared" si="0"/>
-        <v>5.9594864353699855</v>
+        <v>460988.55599470972</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B63" s="1">
-        <v>919611</v>
-      </c>
-      <c r="C63">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" s="5">
+        <v>708245.7</v>
+      </c>
+      <c r="B63" s="5">
+        <v>19338.53</v>
+      </c>
+      <c r="C63" s="5">
+        <v>101958.09994374189</v>
+      </c>
+      <c r="D63" s="5">
+        <v>526252.30000000005</v>
+      </c>
+      <c r="E63" s="5">
+        <v>77489</v>
+      </c>
+      <c r="F63" s="5">
+        <v>390549.3</v>
+      </c>
+      <c r="G63">
         <f t="shared" si="0"/>
-        <v>5.963604157476242</v>
+        <v>463445.30863375531</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B64" s="1">
-        <v>942477</v>
-      </c>
-      <c r="C64">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A64" s="5">
+        <v>712048</v>
+      </c>
+      <c r="B64" s="5">
+        <v>19583.169999999998</v>
+      </c>
+      <c r="C64" s="5">
+        <v>100869.18833727344</v>
+      </c>
+      <c r="D64" s="5">
+        <v>527600.5</v>
+      </c>
+      <c r="E64" s="5">
+        <v>77736.100000000006</v>
+      </c>
+      <c r="F64" s="5">
+        <v>390699.8</v>
+      </c>
+      <c r="G64">
         <f t="shared" si="0"/>
-        <v>5.9742707605807857</v>
+        <v>465472.26006543729</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B65" s="1">
-        <v>956873</v>
-      </c>
-      <c r="C65">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" s="5">
+        <v>715704</v>
+      </c>
+      <c r="B65" s="5">
+        <v>19748.009999999998</v>
+      </c>
+      <c r="C65" s="5">
+        <v>99914.532320105063</v>
+      </c>
+      <c r="D65" s="5">
+        <v>528886.4</v>
+      </c>
+      <c r="E65" s="5">
+        <v>78130.2</v>
+      </c>
+      <c r="F65" s="5">
+        <v>392772.1</v>
+      </c>
+      <c r="G65">
         <f t="shared" si="0"/>
-        <v>5.9808543003063503</v>
+        <v>467589.59606753167</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B66" s="1">
-        <v>969445</v>
-      </c>
-      <c r="C66">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A66" s="5">
+        <v>721992.8</v>
+      </c>
+      <c r="B66" s="5">
+        <v>19720.439999999999</v>
+      </c>
+      <c r="C66" s="5">
+        <v>97415.12416384129</v>
+      </c>
+      <c r="D66" s="5">
+        <v>530535</v>
+      </c>
+      <c r="E66" s="5">
+        <v>78918</v>
+      </c>
+      <c r="F66" s="5">
+        <v>393465.9</v>
+      </c>
+      <c r="G66">
         <f t="shared" si="0"/>
-        <v>5.9865231750711807</v>
+        <v>470824.08140218642</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B67" s="1">
-        <v>971379</v>
-      </c>
-      <c r="C67">
-        <f t="shared" ref="C67:C96" si="1">LOG10(B67)</f>
-        <v>5.9873887103345647</v>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" s="5">
+        <v>723601.4</v>
+      </c>
+      <c r="B67" s="5">
+        <v>19787.349999999999</v>
+      </c>
+      <c r="C67" s="5">
+        <v>98690.803467282662</v>
+      </c>
+      <c r="D67" s="5">
+        <v>529607.1</v>
+      </c>
+      <c r="E67" s="5">
+        <v>78953.3</v>
+      </c>
+      <c r="F67" s="5">
+        <v>394544.5</v>
+      </c>
+      <c r="G67">
+        <f t="shared" ref="G67:G96" si="1">A67*0.518+B67*0.128+C67*0.111+D67*0.086+E67*0.076+F67*0.081</f>
+        <v>471817.75108486839</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B68" s="1">
-        <v>966757</v>
-      </c>
-      <c r="C68">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A68" s="5">
+        <v>726160.6</v>
+      </c>
+      <c r="B68" s="5">
+        <v>19870.72</v>
+      </c>
+      <c r="C68" s="5">
+        <v>100057.7956059663</v>
+      </c>
+      <c r="D68" s="5">
+        <v>530309.19999999995</v>
+      </c>
+      <c r="E68" s="5">
+        <v>79406.8</v>
+      </c>
+      <c r="F68" s="5">
+        <v>397345.8</v>
+      </c>
+      <c r="G68">
         <f t="shared" si="1"/>
-        <v>5.985317325353706</v>
+        <v>473627.57607226225</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B69" s="1">
-        <v>976901</v>
-      </c>
-      <c r="C69">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" s="5">
+        <v>729524.2</v>
+      </c>
+      <c r="B69" s="5">
+        <v>20017.55</v>
+      </c>
+      <c r="C69" s="5">
+        <v>101047.43850352876</v>
+      </c>
+      <c r="D69" s="5">
+        <v>533663.6</v>
+      </c>
+      <c r="E69" s="5">
+        <v>79751.3</v>
+      </c>
+      <c r="F69" s="5">
+        <v>398849.4</v>
+      </c>
+      <c r="G69">
         <f t="shared" si="1"/>
-        <v>5.9898505541668614</v>
+        <v>475935.01747389167</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B70" s="1">
-        <v>1028705</v>
-      </c>
-      <c r="C70">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" s="5">
+        <v>738993.4</v>
+      </c>
+      <c r="B70" s="5">
+        <v>20138.63</v>
+      </c>
+      <c r="C70" s="5">
+        <v>103595.26454659076</v>
+      </c>
+      <c r="D70" s="5">
+        <v>537237.80000000005</v>
+      </c>
+      <c r="E70" s="5">
+        <v>80647.8</v>
+      </c>
+      <c r="F70" s="5">
+        <v>400634.2</v>
+      </c>
+      <c r="G70">
         <f t="shared" si="1"/>
-        <v>6.0122908507193467</v>
+        <v>481658.4540046716</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B71" s="1">
-        <v>1044011</v>
-      </c>
-      <c r="C71">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A71" s="5">
+        <v>744258.4</v>
+      </c>
+      <c r="B71" s="5">
+        <v>20342.689999999999</v>
+      </c>
+      <c r="C71" s="5">
+        <v>107241.74338046882</v>
+      </c>
+      <c r="D71" s="5">
+        <v>541349.1</v>
+      </c>
+      <c r="E71" s="5">
+        <v>80893.600000000006</v>
+      </c>
+      <c r="F71" s="5">
+        <v>402189</v>
+      </c>
+      <c r="G71">
         <f t="shared" si="1"/>
-        <v>6.0187050745418507</v>
+        <v>485314.79423523205</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B72" s="1">
-        <v>1044442</v>
-      </c>
-      <c r="C72">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A72" s="5">
+        <v>750181.4</v>
+      </c>
+      <c r="B72" s="5">
+        <v>20468.53</v>
+      </c>
+      <c r="C72" s="5">
+        <v>107753.36449256641</v>
+      </c>
+      <c r="D72" s="5">
+        <v>545208.80000000005</v>
+      </c>
+      <c r="E72" s="5">
+        <v>81343.399999999994</v>
+      </c>
+      <c r="F72" s="5">
+        <v>402874.7</v>
+      </c>
+      <c r="G72">
         <f t="shared" si="1"/>
-        <v>6.0188843277252904</v>
+        <v>488877.46639867494</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B73" s="1">
-        <v>1061049</v>
-      </c>
-      <c r="C73">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A73" s="5">
+        <v>757786.3</v>
+      </c>
+      <c r="B73" s="5">
+        <v>20732.849999999999</v>
+      </c>
+      <c r="C73" s="5">
+        <v>109943.57544539485</v>
+      </c>
+      <c r="D73" s="5">
+        <v>548493.69999999995</v>
+      </c>
+      <c r="E73" s="5">
+        <v>81740.2</v>
+      </c>
+      <c r="F73" s="5">
+        <v>405278.4</v>
+      </c>
+      <c r="G73">
         <f t="shared" si="1"/>
-        <v>6.0257354403935492</v>
+        <v>493601.10887443885</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B74" s="1">
-        <v>1077616</v>
-      </c>
-      <c r="C74">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A74" s="5">
+        <v>753599.8</v>
+      </c>
+      <c r="B74" s="5">
+        <v>20928.099999999999</v>
+      </c>
+      <c r="C74" s="5">
+        <v>113544.05149310874</v>
+      </c>
+      <c r="D74" s="5">
+        <v>548281.59999999998</v>
+      </c>
+      <c r="E74" s="5">
+        <v>82176</v>
+      </c>
+      <c r="F74" s="5">
+        <v>404562.1</v>
+      </c>
+      <c r="G74">
         <f t="shared" si="1"/>
-        <v>6.0324640309889865</v>
+        <v>491814.00661573501</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B75" s="1">
-        <v>1077052</v>
-      </c>
-      <c r="C75">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A75" s="5">
+        <v>759522.8</v>
+      </c>
+      <c r="B75" s="5">
+        <v>21195.49</v>
+      </c>
+      <c r="C75" s="5">
+        <v>112958.35581728176</v>
+      </c>
+      <c r="D75" s="5">
+        <v>549730.19999999995</v>
+      </c>
+      <c r="E75" s="5">
+        <v>82900.2</v>
+      </c>
+      <c r="F75" s="5">
+        <v>405398</v>
+      </c>
+      <c r="G75">
         <f t="shared" si="1"/>
-        <v>6.0322366715132922</v>
+        <v>495098.66101571824</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B76" s="1">
-        <v>1080844</v>
-      </c>
-      <c r="C76">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A76" s="5">
+        <v>754550.4</v>
+      </c>
+      <c r="B76" s="5">
+        <v>21400.52</v>
+      </c>
+      <c r="C76" s="5">
+        <v>113298.87060791969</v>
+      </c>
+      <c r="D76" s="5">
+        <v>552359.30000000005</v>
+      </c>
+      <c r="E76" s="5">
+        <v>83308.7</v>
+      </c>
+      <c r="F76" s="5">
+        <v>405381.9</v>
+      </c>
+      <c r="G76">
         <f t="shared" si="1"/>
-        <v>6.0337630160364073</v>
+        <v>492842.84329747915</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B77" s="1">
-        <v>1097264</v>
-      </c>
-      <c r="C77">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A77" s="5">
+        <v>757914.1</v>
+      </c>
+      <c r="B77" s="5">
+        <v>21433.47</v>
+      </c>
+      <c r="C77" s="5">
+        <v>114509.33872956064</v>
+      </c>
+      <c r="D77" s="5">
+        <v>556528.30000000005</v>
+      </c>
+      <c r="E77" s="5">
+        <v>84061.4</v>
+      </c>
+      <c r="F77" s="5">
+        <v>406587.9</v>
+      </c>
+      <c r="G77">
         <f t="shared" si="1"/>
-        <v>6.0403111307190693</v>
+        <v>495237.24465898122</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B78" s="1">
-        <v>1092153</v>
-      </c>
-      <c r="C78">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A78" s="5">
+        <v>762886.4</v>
+      </c>
+      <c r="B78" s="5">
+        <v>21734.84</v>
+      </c>
+      <c r="C78" s="5">
+        <v>116109.07569276549</v>
+      </c>
+      <c r="D78" s="5">
+        <v>561652.80000000005</v>
+      </c>
+      <c r="E78" s="5">
+        <v>84697</v>
+      </c>
+      <c r="F78" s="5">
+        <v>407464.2</v>
+      </c>
+      <c r="G78">
         <f t="shared" si="1"/>
-        <v>6.0382834830584811</v>
+        <v>498589.035121897</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B79" s="1">
-        <v>1103182</v>
-      </c>
-      <c r="C79">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A79" s="5">
+        <v>763325.1</v>
+      </c>
+      <c r="B79" s="5">
+        <v>21689.65</v>
+      </c>
+      <c r="C79" s="5">
+        <v>117716.39072461061</v>
+      </c>
+      <c r="D79" s="5">
+        <v>564746.19999999995</v>
+      </c>
+      <c r="E79" s="5">
+        <v>84498.4</v>
+      </c>
+      <c r="F79" s="5">
+        <v>408589.4</v>
+      </c>
+      <c r="G79">
         <f t="shared" si="1"/>
-        <v>6.0426471670868933</v>
+        <v>499330.98937043175</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B80" s="1">
-        <v>1108610</v>
-      </c>
-      <c r="C80">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A80" s="5">
+        <v>766250.1</v>
+      </c>
+      <c r="B80" s="5">
+        <v>21693.77</v>
+      </c>
+      <c r="C80" s="5">
+        <v>117650.51871063358</v>
+      </c>
+      <c r="D80" s="5">
+        <v>564699.4</v>
+      </c>
+      <c r="E80" s="5">
+        <v>84708.5</v>
+      </c>
+      <c r="F80" s="5">
+        <v>407077.4</v>
+      </c>
+      <c r="G80">
         <f t="shared" si="1"/>
-        <v>6.0447787917426696</v>
+        <v>500728.82573688036</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B81" s="1">
-        <v>1087679</v>
-      </c>
-      <c r="C81">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A81" s="5">
+        <v>763690.8</v>
+      </c>
+      <c r="B81" s="5">
+        <v>21770.41</v>
+      </c>
+      <c r="C81" s="5">
+        <v>119355.13517296076</v>
+      </c>
+      <c r="D81" s="5">
+        <v>561937.1</v>
+      </c>
+      <c r="E81" s="5">
+        <v>84406.8</v>
+      </c>
+      <c r="F81" s="5">
+        <v>405563.4</v>
+      </c>
+      <c r="G81">
         <f t="shared" si="1"/>
-        <v>6.0365007436176228</v>
+        <v>499219.00968419871</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B82" s="1">
-        <v>1045667</v>
-      </c>
-      <c r="C82">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A82" s="5">
+        <v>748188.8</v>
+      </c>
+      <c r="B82" s="5">
+        <v>21507.3</v>
+      </c>
+      <c r="C82" s="5">
+        <v>119045.72049675077</v>
+      </c>
+      <c r="D82" s="5">
+        <v>533413.9</v>
+      </c>
+      <c r="E82" s="5">
+        <v>82501.899999999994</v>
+      </c>
+      <c r="F82" s="5">
+        <v>381973.9</v>
+      </c>
+      <c r="G82">
         <f t="shared" si="1"/>
-        <v>6.0193934024206754</v>
+        <v>486612.43347513938</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B83" s="1">
-        <v>821963</v>
-      </c>
-      <c r="C83">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A83" s="5">
+        <v>681793.6</v>
+      </c>
+      <c r="B83" s="5">
+        <v>19775.22</v>
+      </c>
+      <c r="C83" s="5">
+        <v>104037.33315566217</v>
+      </c>
+      <c r="D83" s="5">
+        <v>468366.4</v>
+      </c>
+      <c r="E83" s="5">
+        <v>72665.600000000006</v>
+      </c>
+      <c r="F83" s="5">
+        <v>334885.2</v>
+      </c>
+      <c r="G83">
         <f t="shared" si="1"/>
-        <v>5.9148522685650029</v>
+        <v>440176.25414027856</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B84" s="1">
-        <v>1052320</v>
-      </c>
-      <c r="C84">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A84" s="5">
+        <v>740949.7</v>
+      </c>
+      <c r="B84" s="5">
+        <v>21640.71</v>
+      </c>
+      <c r="C84" s="5">
+        <v>112404.45365095805</v>
+      </c>
+      <c r="D84" s="5">
+        <v>540285.19999999995</v>
+      </c>
+      <c r="E84" s="5">
+        <v>81034.100000000006</v>
+      </c>
+      <c r="F84" s="5">
+        <v>383135.4</v>
+      </c>
+      <c r="G84">
         <f t="shared" si="1"/>
-        <v>6.0221478245151809</v>
+        <v>482715.93603525637</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B85" s="1">
-        <v>1115561</v>
-      </c>
-      <c r="C85">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A85" s="5">
+        <v>748115.7</v>
+      </c>
+      <c r="B85" s="5">
+        <v>21749.59</v>
+      </c>
+      <c r="C85" s="5">
+        <v>110970.89964706666</v>
+      </c>
+      <c r="D85" s="5">
+        <v>539664.19999999995</v>
+      </c>
+      <c r="E85" s="5">
+        <v>80013.399999999994</v>
+      </c>
+      <c r="F85" s="5">
+        <v>382900.3</v>
+      </c>
+      <c r="G85">
         <f t="shared" si="1"/>
-        <v>6.0474933229292063</v>
+        <v>486132.71388082439</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B86" s="1">
-        <v>1092274</v>
-      </c>
-      <c r="C86">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A86" s="5">
+        <v>743509</v>
+      </c>
+      <c r="B86" s="5">
+        <v>22090.58</v>
+      </c>
+      <c r="C86" s="5">
+        <v>112559.09980861034</v>
+      </c>
+      <c r="D86" s="5">
+        <v>541862.6</v>
+      </c>
+      <c r="E86" s="5">
+        <v>78811.100000000006</v>
+      </c>
+      <c r="F86" s="5">
+        <v>389680.9</v>
+      </c>
+      <c r="G86">
         <f t="shared" si="1"/>
-        <v>6.0383315960257393</v>
+        <v>484613.29641875572</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B87" s="1">
-        <v>1096656</v>
-      </c>
-      <c r="C87">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A87" s="5">
+        <v>760985.2</v>
+      </c>
+      <c r="B87" s="5">
+        <v>22319.64</v>
+      </c>
+      <c r="C87" s="5">
+        <v>115843.03724801837</v>
+      </c>
+      <c r="D87" s="5">
+        <v>548463.69999999995</v>
+      </c>
+      <c r="E87" s="5">
+        <v>82423.8</v>
+      </c>
+      <c r="F87" s="5">
+        <v>399237.6</v>
+      </c>
+      <c r="G87">
         <f t="shared" si="1"/>
-        <v>6.0400704190689112</v>
+        <v>495676.15725453012</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B88" s="1">
-        <v>1048014</v>
-      </c>
-      <c r="C88">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A88" s="5">
+        <v>761643.3</v>
+      </c>
+      <c r="B88" s="5">
+        <v>22461.52</v>
+      </c>
+      <c r="C88" s="5">
+        <v>117271.2161363089</v>
+      </c>
+      <c r="D88" s="5">
+        <v>564825.19999999995</v>
+      </c>
+      <c r="E88" s="5">
+        <v>85414.399999999994</v>
+      </c>
+      <c r="F88" s="5">
+        <v>409157.8</v>
+      </c>
+      <c r="G88">
         <f t="shared" si="1"/>
-        <v>6.0203670842527988</v>
+        <v>498631.65235113032</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B89" s="1">
-        <v>1071971</v>
-      </c>
-      <c r="C89">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A89" s="5">
+        <v>765738.2</v>
+      </c>
+      <c r="B89" s="5">
+        <v>22573.4</v>
+      </c>
+      <c r="C89" s="5">
+        <v>118284.97173672925</v>
+      </c>
+      <c r="D89" s="5">
+        <v>568002.6</v>
+      </c>
+      <c r="E89" s="5">
+        <v>85429.1</v>
+      </c>
+      <c r="F89" s="5">
+        <v>415435.4</v>
+      </c>
+      <c r="G89">
         <f t="shared" si="1"/>
-        <v>6.0301830365597979</v>
+        <v>501662.51726277702</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B90" s="1">
-        <v>1117383</v>
-      </c>
-      <c r="C90">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A90" s="5">
+        <v>770929.9</v>
+      </c>
+      <c r="B90" s="5">
+        <v>22496.65</v>
+      </c>
+      <c r="C90" s="5">
+        <v>122041.4449491672</v>
+      </c>
+      <c r="D90" s="5">
+        <v>567496.6</v>
+      </c>
+      <c r="E90" s="5">
+        <v>85692.800000000003</v>
+      </c>
+      <c r="F90" s="5">
+        <v>418471.4</v>
+      </c>
+      <c r="G90">
         <f t="shared" si="1"/>
-        <v>6.0482020596656749</v>
+        <v>504981.40358935756</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B91" s="1">
-        <v>1133299</v>
-      </c>
-      <c r="C91">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A91" s="5">
+        <v>772099.8</v>
+      </c>
+      <c r="B91" s="5">
+        <v>22388.639999999999</v>
+      </c>
+      <c r="C91" s="5">
+        <v>120033.69191049914</v>
+      </c>
+      <c r="D91" s="5">
+        <v>569946.9</v>
+      </c>
+      <c r="E91" s="5">
+        <v>88114.7</v>
+      </c>
+      <c r="F91" s="5">
+        <v>424594.8</v>
+      </c>
+      <c r="G91">
         <f t="shared" si="1"/>
-        <v>6.0543445055551768</v>
+        <v>506241.51152206544</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B92" s="1">
-        <v>1181567</v>
-      </c>
-      <c r="C92">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A92" s="5">
+        <v>774366.6</v>
+      </c>
+      <c r="B92" s="5">
+        <v>22474.17</v>
+      </c>
+      <c r="C92" s="5">
+        <v>118256.80376077747</v>
+      </c>
+      <c r="D92" s="5">
+        <v>572890.9</v>
+      </c>
+      <c r="E92" s="5">
+        <v>88033.7</v>
+      </c>
+      <c r="F92" s="5">
+        <v>425682.9</v>
+      </c>
+      <c r="G92">
         <f t="shared" si="1"/>
-        <v>6.0724583530570779</v>
+        <v>507564.59127744631</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B93" s="1">
-        <v>1188505</v>
-      </c>
-      <c r="C93">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A93" s="5">
+        <v>771661.1</v>
+      </c>
+      <c r="B93" s="5">
+        <v>22545.24</v>
+      </c>
+      <c r="C93" s="5">
+        <v>116733.53217413377</v>
+      </c>
+      <c r="D93" s="5">
+        <v>575088.69999999995</v>
+      </c>
+      <c r="E93" s="5">
+        <v>88046.7</v>
+      </c>
+      <c r="F93" s="5">
+        <v>425031</v>
+      </c>
+      <c r="G93">
         <f t="shared" si="1"/>
-        <v>6.075001013130116</v>
+        <v>506140.35099132883</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B94" s="1">
-        <v>1189257</v>
-      </c>
-      <c r="C94">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A94" s="5">
+        <v>768023.3</v>
+      </c>
+      <c r="B94" s="5">
+        <v>22700.34</v>
+      </c>
+      <c r="C94" s="5">
+        <v>118384.86863065782</v>
+      </c>
+      <c r="D94" s="5">
+        <v>575446.6</v>
+      </c>
+      <c r="E94" s="5">
+        <v>87465.4</v>
+      </c>
+      <c r="F94" s="5">
+        <v>426964.9</v>
+      </c>
+      <c r="G94">
         <f t="shared" si="1"/>
-        <v>6.0752757163689424</v>
+        <v>504602.36823800305</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B95" s="1">
-        <v>1189464</v>
-      </c>
-      <c r="C95">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A95" s="5">
+        <v>767438.2</v>
+      </c>
+      <c r="B95" s="5">
+        <v>22926.32</v>
+      </c>
+      <c r="C95" s="5">
+        <v>122099.17118546928</v>
+      </c>
+      <c r="D95" s="5">
+        <v>580546.6</v>
+      </c>
+      <c r="E95" s="5">
+        <v>87092.4</v>
+      </c>
+      <c r="F95" s="5">
+        <v>426273.1</v>
+      </c>
+      <c r="G95">
         <f t="shared" si="1"/>
-        <v>6.0753513023312991</v>
+        <v>505094.71566158708</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B96" s="1">
-        <v>1175068</v>
-      </c>
-      <c r="C96">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A96" s="5">
+        <v>767438.3</v>
+      </c>
+      <c r="B96" s="5">
+        <v>23045.9</v>
+      </c>
+      <c r="C96" s="5">
+        <v>125425.05334281651</v>
+      </c>
+      <c r="D96" s="5">
+        <v>581949.1</v>
+      </c>
+      <c r="E96" s="5">
+        <v>86412.4</v>
+      </c>
+      <c r="F96" s="5">
+        <v>426811.8</v>
+      </c>
+      <c r="G96">
         <f t="shared" si="1"/>
-        <v>6.0700629995186137</v>
+        <v>505591.81632105267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>